<commit_message>
cambios en get global dni
</commit_message>
<xml_diff>
--- a/Datos IA.xlsx
+++ b/Datos IA.xlsx
@@ -1980,7 +1980,16 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2525,7 +2534,7 @@
       </c>
       <c r="I10"/>
     </row>
-    <row r="11" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="32">
         <v>1994</v>
       </c>
@@ -2549,7 +2558,7 @@
       </c>
       <c r="I11"/>
     </row>
-    <row r="12" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="32">
         <v>2001</v>
       </c>
@@ -2621,7 +2630,7 @@
       </c>
       <c r="I14"/>
     </row>
-    <row r="15" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="39">
         <v>26</v>
       </c>
@@ -2645,7 +2654,7 @@
       </c>
       <c r="I15"/>
     </row>
-    <row r="16" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="32">
         <v>1990</v>
       </c>
@@ -4445,7 +4454,7 @@
       </c>
       <c r="I90"/>
     </row>
-    <row r="91" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="32">
         <v>1991</v>
       </c>
@@ -4685,7 +4694,7 @@
       </c>
       <c r="I100"/>
     </row>
-    <row r="101" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="32">
         <v>2003</v>
       </c>
@@ -4757,7 +4766,7 @@
       </c>
       <c r="I103"/>
     </row>
-    <row r="104" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="32">
         <v>2004</v>
       </c>
@@ -5045,7 +5054,7 @@
       </c>
       <c r="I115"/>
     </row>
-    <row r="116" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="32">
         <v>1996</v>
       </c>
@@ -5717,7 +5726,7 @@
       </c>
       <c r="I143"/>
     </row>
-    <row r="144" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="32">
         <v>1992</v>
       </c>
@@ -5741,7 +5750,7 @@
       </c>
       <c r="I144"/>
     </row>
-    <row r="145" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="32">
         <v>2000</v>
       </c>
@@ -6557,7 +6566,7 @@
       </c>
       <c r="I178"/>
     </row>
-    <row r="179" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="32">
         <v>1993</v>
       </c>
@@ -7997,7 +8006,7 @@
       </c>
       <c r="I238"/>
     </row>
-    <row r="239" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="32">
         <v>1999</v>
       </c>
@@ -8525,7 +8534,7 @@
       </c>
       <c r="I260"/>
     </row>
-    <row r="261" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A261" s="32">
         <v>1997</v>
       </c>
@@ -9701,7 +9710,7 @@
       </c>
       <c r="I309"/>
     </row>
-    <row r="310" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A310" s="32">
         <v>1995</v>
       </c>
@@ -10325,7 +10334,7 @@
       </c>
       <c r="I335"/>
     </row>
-    <row r="336" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A336" s="39">
         <v>25</v>
       </c>
@@ -10997,7 +11006,7 @@
       </c>
       <c r="I363"/>
     </row>
-    <row r="364" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A364" s="22">
         <v>1870</v>
       </c>
@@ -11669,7 +11678,7 @@
       </c>
       <c r="I391"/>
     </row>
-    <row r="392" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A392" s="32">
         <v>1989</v>
       </c>
@@ -11837,7 +11846,7 @@
       </c>
       <c r="I398"/>
     </row>
-    <row r="399" spans="1:9" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A399" s="32">
         <v>1998</v>
       </c>
@@ -12437,7 +12446,7 @@
       </c>
       <c r="I423"/>
     </row>
-    <row r="424" spans="1:9" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A424" s="32">
         <v>1988</v>
       </c>
@@ -13646,9 +13655,7 @@
   </sheetData>
   <autoFilter ref="A1:G442">
     <filterColumn colId="1">
-      <filters>
-        <filter val="ROVERE MATEO JOSE"/>
-      </filters>
+      <colorFilter dxfId="0"/>
     </filterColumn>
     <sortState ref="A2:G444">
       <sortCondition ref="B1:B424"/>
@@ -13662,7 +13669,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>'[Headcount para IA.xlsx]Hoja1'!#REF!</xm:f>
+            <xm:f>'C:\Users\virginia.carrizo\Downloads\[Headcount para IA.xlsx]Hoja1'!#REF!</xm:f>
           </x14:formula1>
           <xm:sqref>G423:G442</xm:sqref>
         </x14:dataValidation>

</xml_diff>